<commit_message>
minor updates to preso
</commit_message>
<xml_diff>
--- a/Corpus/descriptive_analysis/tables/oa_status.xlsx
+++ b/Corpus/descriptive_analysis/tables/oa_status.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,11 @@
           <t>Count</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Percentage</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -452,6 +457,9 @@
       <c r="C2" t="n">
         <v>2360</v>
       </c>
+      <c r="D2" t="n">
+        <v>38.59362224039248</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -465,6 +473,9 @@
       <c r="C3" t="n">
         <v>1167</v>
       </c>
+      <c r="D3" t="n">
+        <v>19.08421913327882</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -478,6 +489,9 @@
       <c r="C4" t="n">
         <v>1091</v>
       </c>
+      <c r="D4" t="n">
+        <v>17.84137367130008</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -491,6 +505,9 @@
       <c r="C5" t="n">
         <v>761</v>
       </c>
+      <c r="D5" t="n">
+        <v>12.44480784955029</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -504,6 +521,9 @@
       <c r="C6" t="n">
         <v>688</v>
       </c>
+      <c r="D6" t="n">
+        <v>11.25102207686018</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -516,6 +536,9 @@
       </c>
       <c r="C7" t="n">
         <v>48</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.7849550286181521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>